<commit_message>
Mise à jour automatique des résultats FFBB
</commit_message>
<xml_diff>
--- a/data/rencontres/rencontres.xlsx
+++ b/data/rencontres/rencontres.xlsx
@@ -50,123 +50,123 @@
     <t>Forfait 2</t>
   </si>
   <si>
+    <t>AMIU15M</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (1) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">CARNIERES BC (2) </t>
+  </si>
+  <si>
+    <t>04/09/2026</t>
+  </si>
+  <si>
+    <t>19:00</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Non</t>
+  </si>
+  <si>
+    <t>AMIU9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TEMPLEUVE L P (2) </t>
+  </si>
+  <si>
+    <t>05/09/2026</t>
+  </si>
+  <si>
+    <t>10:30</t>
+  </si>
+  <si>
+    <t>AMIU13M</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (6) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AULNOY VALENCIENNES S (7) </t>
+  </si>
+  <si>
+    <t>06/09/2026</t>
+  </si>
+  <si>
+    <t>09:30</t>
+  </si>
+  <si>
+    <t>AMISM</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (13) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">OSTREVENT BASKET BALL EAA MONCHECOURT (15) </t>
+  </si>
+  <si>
+    <t>20:30</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>09:00</t>
+  </si>
+  <si>
+    <t>AMILOISIRS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BASKET CLUB HULLUCH (2) </t>
+  </si>
+  <si>
+    <t>11:00</t>
+  </si>
+  <si>
+    <t>AMIU11M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (7) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ONNAING JA (8) </t>
+  </si>
+  <si>
+    <t>13:30</t>
+  </si>
+  <si>
+    <t>AMIU18M</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (8) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNION DECHY SIN BASKET (9) </t>
+  </si>
+  <si>
+    <t>13:00</t>
+  </si>
+  <si>
     <t>AMIU18F</t>
   </si>
   <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (8) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNION DECHY SIN BASKET (9) </t>
-  </si>
-  <si>
-    <t>05/09/2026</t>
-  </si>
-  <si>
     <t>20:00</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
-    <t>Non</t>
-  </si>
-  <si>
-    <t>AMIU18M</t>
-  </si>
-  <si>
-    <t>06/09/2026</t>
-  </si>
-  <si>
-    <t>13:00</t>
-  </si>
-  <si>
-    <t>AMIU15M</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (1) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">CARNIERES BC (2) </t>
-  </si>
-  <si>
-    <t>04/09/2026</t>
-  </si>
-  <si>
-    <t>19:00</t>
-  </si>
-  <si>
-    <t>AMIU13M</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (6) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">AULNOY VALENCIENNES S (7) </t>
-  </si>
-  <si>
-    <t>09:30</t>
-  </si>
-  <si>
-    <t>AMISM</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (13) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">OSTREVENT BASKET BALL EAA MONCHECOURT (15) </t>
-  </si>
-  <si>
-    <t>20:30</t>
-  </si>
-  <si>
-    <t>AMIU9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TEMPLEUVE L P (2) </t>
-  </si>
-  <si>
-    <t>10:30</t>
-  </si>
-  <si>
-    <t>2</t>
-  </si>
-  <si>
-    <t>09:00</t>
-  </si>
-  <si>
-    <t>AMILOISIRS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BASKET CLUB HULLUCH (2) </t>
-  </si>
-  <si>
-    <t>11:00</t>
-  </si>
-  <si>
-    <t>AMIU11M</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (7) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">ONNAING JA (8) </t>
-  </si>
-  <si>
-    <t>13:30</t>
-  </si>
-  <si>
     <t>AMIU15F</t>
   </si>
   <si>
@@ -188,16 +188,16 @@
     <t>15:00</t>
   </si>
   <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THIANT BC (14) </t>
+  </si>
+  <si>
     <t xml:space="preserve">ANNOEULLIN B C (9) </t>
   </si>
   <si>
     <t>12:00</t>
-  </si>
-  <si>
-    <t>10</t>
-  </si>
-  <si>
-    <t xml:space="preserve">THIANT BC (14) </t>
   </si>
 </sst>
 </file>
@@ -345,13 +345,13 @@
         <v>14</v>
       </c>
       <c r="D3" t="s" s="0">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="E3" t="s" s="0">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F3" t="s" s="0">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G3" s="0"/>
       <c r="H3" t="s" s="0">
@@ -372,22 +372,22 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="0">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C4" t="s" s="0">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D4" t="s" s="0">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E4" t="s" s="0">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F4" t="s" s="0">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G4" s="0"/>
       <c r="H4" t="s" s="0">
@@ -408,22 +408,22 @@
     </row>
     <row r="5">
       <c r="A5" t="s" s="0">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s" s="0">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C5" t="s" s="0">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D5" t="s" s="0">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="F5" t="s" s="0">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G5" s="0"/>
       <c r="H5" t="s" s="0">
@@ -444,22 +444,22 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s" s="0">
         <v>35</v>
       </c>
       <c r="C6" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="D6" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="E6" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="F6" t="s" s="0">
         <v>36</v>
-      </c>
-      <c r="D6" t="s" s="0">
-        <v>37</v>
-      </c>
-      <c r="E6" t="s" s="0">
-        <v>27</v>
-      </c>
-      <c r="F6" t="s" s="0">
-        <v>38</v>
       </c>
       <c r="G6" s="0"/>
       <c r="H6" t="s" s="0">
@@ -480,22 +480,22 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="D7" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="E7" t="s" s="0">
+        <v>28</v>
+      </c>
+      <c r="F7" t="s" s="0">
         <v>39</v>
-      </c>
-      <c r="B7" t="s" s="0">
-        <v>24</v>
-      </c>
-      <c r="C7" t="s" s="0">
-        <v>25</v>
-      </c>
-      <c r="D7" t="s" s="0">
-        <v>40</v>
-      </c>
-      <c r="E7" t="s" s="0">
-        <v>16</v>
-      </c>
-      <c r="F7" t="s" s="0">
-        <v>41</v>
       </c>
       <c r="G7" s="0"/>
       <c r="H7" t="s" s="0">
@@ -516,19 +516,19 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="D8" t="s" s="0">
         <v>42</v>
       </c>
-      <c r="C8" t="s" s="0">
-        <v>25</v>
-      </c>
-      <c r="D8" t="s" s="0">
-        <v>40</v>
-      </c>
       <c r="E8" t="s" s="0">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F8" t="s" s="0">
         <v>43</v>
@@ -555,19 +555,19 @@
         <v>44</v>
       </c>
       <c r="B9" t="s" s="0">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>25</v>
+        <v>46</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>21</v>
+        <v>28</v>
       </c>
       <c r="F9" t="s" s="0">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G9" s="0"/>
       <c r="H9" t="s" s="0">
@@ -588,19 +588,19 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
+        <v>49</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="D10" t="s" s="0">
         <v>47</v>
       </c>
-      <c r="B10" t="s" s="0">
-        <v>30</v>
-      </c>
-      <c r="C10" t="s" s="0">
-        <v>48</v>
-      </c>
-      <c r="D10" t="s" s="0">
-        <v>49</v>
-      </c>
       <c r="E10" t="s" s="0">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F10" t="s" s="0">
         <v>50</v>
@@ -627,16 +627,16 @@
         <v>51</v>
       </c>
       <c r="B11" t="s" s="0">
-        <v>13</v>
+        <v>45</v>
       </c>
       <c r="C11" t="s" s="0">
-        <v>48</v>
+        <v>41</v>
       </c>
       <c r="D11" t="s" s="0">
         <v>52</v>
       </c>
       <c r="E11" t="s" s="0">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F11" t="s" s="0">
         <v>53</v>
@@ -663,7 +663,7 @@
         <v>54</v>
       </c>
       <c r="B12" t="s" s="0">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="C12" t="s" s="0">
         <v>55</v>
@@ -672,7 +672,7 @@
         <v>56</v>
       </c>
       <c r="E12" t="s" s="0">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="F12" t="s" s="0">
         <v>57</v>
@@ -696,22 +696,22 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="0">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="B13" t="s" s="0">
-        <v>13</v>
+        <v>58</v>
       </c>
       <c r="C13" t="s" s="0">
-        <v>48</v>
+        <v>32</v>
       </c>
       <c r="D13" t="s" s="0">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E13" t="s" s="0">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="F13" t="s" s="0">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="G13" s="0"/>
       <c r="H13" t="s" s="0">
@@ -732,22 +732,22 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="0">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B14" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="D14" t="s" s="0">
         <v>60</v>
       </c>
-      <c r="C14" t="s" s="0">
-        <v>36</v>
-      </c>
-      <c r="D14" t="s" s="0">
+      <c r="E14" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="F14" t="s" s="0">
         <v>61</v>
-      </c>
-      <c r="E14" t="s" s="0">
-        <v>21</v>
-      </c>
-      <c r="F14" t="s" s="0">
-        <v>57</v>
       </c>
       <c r="G14" s="0"/>
       <c r="H14" t="s" s="0">

</xml_diff>

<commit_message>
Update doc et videos
</commit_message>
<xml_diff>
--- a/data/rencontres/rencontres.xlsx
+++ b/data/rencontres/rencontres.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="77">
   <si>
     <t>Division</t>
   </si>
@@ -50,60 +50,78 @@
     <t>Forfait 2</t>
   </si>
   <si>
+    <t>AMILOISIRS</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (1) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">BASKET CLUB HULLUCH (2) </t>
+  </si>
+  <si>
+    <t>06/09/2026</t>
+  </si>
+  <si>
+    <t>11:00</t>
+  </si>
+  <si>
+    <t>THF8X6GZ</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Non</t>
+  </si>
+  <si>
     <t>AMIU11M</t>
   </si>
   <si>
     <t>4</t>
   </si>
   <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (8) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">ONNAING JA (9) </t>
+  </si>
+  <si>
+    <t>05/09/2026</t>
+  </si>
+  <si>
+    <t>13:30</t>
+  </si>
+  <si>
+    <t>A2TVWMAZ</t>
+  </si>
+  <si>
+    <t>AMIU15M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CARNIERES BC (2) </t>
+  </si>
+  <si>
+    <t>04/09/2026</t>
+  </si>
+  <si>
+    <t>19:00</t>
+  </si>
+  <si>
+    <t>Y3863HXE</t>
+  </si>
+  <si>
+    <t>AMIU15F</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
     <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (7) </t>
   </si>
   <si>
-    <t xml:space="preserve">ONNAING JA (8) </t>
-  </si>
-  <si>
-    <t>05/09/2026</t>
-  </si>
-  <si>
-    <t>13:30</t>
-  </si>
-  <si>
-    <t>A2TVWMAZ</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>Non</t>
-  </si>
-  <si>
-    <t>AMIU15M</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (1) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">CARNIERES BC (2) </t>
-  </si>
-  <si>
-    <t>04/09/2026</t>
-  </si>
-  <si>
-    <t>19:00</t>
-  </si>
-  <si>
-    <t>Y3863HXE</t>
-  </si>
-  <si>
-    <t>AMIU15F</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
     <t xml:space="preserve">BASKET CLUB PEVELE (8) </t>
   </si>
   <si>
@@ -131,7 +149,7 @@
     <t>FYAVJ6FE</t>
   </si>
   <si>
-    <t xml:space="preserve">ANNOEULLIN B C (9) </t>
+    <t xml:space="preserve">ANNOEULLIN B C (10) </t>
   </si>
   <si>
     <t>12:00</t>
@@ -143,21 +161,69 @@
     <t>AMISM</t>
   </si>
   <si>
+    <t>10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (15) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">THIANT BC (16) </t>
+  </si>
+  <si>
+    <t>JEAN DEGROS</t>
+  </si>
+  <si>
+    <t>ZUKWCAJX</t>
+  </si>
+  <si>
+    <t>AMIU18F</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (10) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">UNION DECHY SIN BASKET (11) </t>
+  </si>
+  <si>
+    <t>20:00</t>
+  </si>
+  <si>
+    <t>87XPKJA7</t>
+  </si>
+  <si>
+    <t>AMIU18M</t>
+  </si>
+  <si>
+    <t>13:00</t>
+  </si>
+  <si>
+    <t>L3XF6NMK</t>
+  </si>
+  <si>
+    <t>AMIU13M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (6) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">AULNOY VALENCIENNES S (7) </t>
+  </si>
+  <si>
+    <t>09:30</t>
+  </si>
+  <si>
+    <t>97EDTAHL</t>
+  </si>
+  <si>
     <t>11</t>
   </si>
   <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (14) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">OSTREVENT BASKET BALL EAA MONCHECOURT (16) </t>
+    <t xml:space="preserve">OSTREVENT BASKET BALL EAA MONCHECOURT (17) </t>
   </si>
   <si>
     <t>20:30</t>
   </si>
   <si>
-    <t>JEAN DEGROS</t>
-  </si>
-  <si>
     <t>EZJX8MF7</t>
   </si>
   <si>
@@ -177,21 +243,6 @@
   </si>
   <si>
     <t>32CMFD7W</t>
-  </si>
-  <si>
-    <t>AMIU18F</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AMICALE BASKET PECQUENCOURT (9) </t>
-  </si>
-  <si>
-    <t xml:space="preserve">UNION DECHY SIN BASKET (10) </t>
-  </si>
-  <si>
-    <t>20:00</t>
-  </si>
-  <si>
-    <t>87XPKJA7</t>
   </si>
 </sst>
 </file>
@@ -237,10 +288,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:L14"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="8.296875" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="9.91796875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="11.29296875" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="32.32421875" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="42.3671875" customWidth="true" bestFit="true"/>
@@ -369,16 +420,16 @@
         <v>28</v>
       </c>
       <c r="B4" t="s" s="0">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s" s="0">
         <v>14</v>
       </c>
       <c r="D4" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="E4" t="s" s="0">
         <v>30</v>
-      </c>
-      <c r="E4" t="s" s="0">
-        <v>16</v>
       </c>
       <c r="F4" t="s" s="0">
         <v>31</v>
@@ -414,7 +465,7 @@
         <v>36</v>
       </c>
       <c r="E5" t="s" s="0">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="F5" t="s" s="0">
         <v>37</v>
@@ -438,26 +489,26 @@
     </row>
     <row r="6">
       <c r="A6" t="s" s="0">
-        <v>12</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s" s="0">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="C6" t="s" s="0">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="D6" t="s" s="0">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="E6" t="s" s="0">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="F6" t="s" s="0">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="G6" s="0"/>
       <c r="H6" t="s" s="0">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="I6" t="s" s="0">
         <v>19</v>
@@ -474,13 +525,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s" s="0">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="B7" t="s" s="0">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="C7" t="s" s="0">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="D7" t="s" s="0">
         <v>45</v>
@@ -491,11 +542,9 @@
       <c r="F7" t="s" s="0">
         <v>46</v>
       </c>
-      <c r="G7" t="s" s="0">
+      <c r="G7" s="0"/>
+      <c r="H7" t="s" s="0">
         <v>47</v>
-      </c>
-      <c r="H7" t="s" s="0">
-        <v>48</v>
       </c>
       <c r="I7" t="s" s="0">
         <v>19</v>
@@ -512,26 +561,28 @@
     </row>
     <row r="8">
       <c r="A8" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="B8" t="s" s="0">
         <v>49</v>
       </c>
-      <c r="B8" t="s" s="0">
-        <v>22</v>
-      </c>
       <c r="C8" t="s" s="0">
-        <v>23</v>
+        <v>50</v>
       </c>
       <c r="D8" t="s" s="0">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E8" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F8" t="s" s="0">
-        <v>51</v>
-      </c>
-      <c r="G8" s="0"/>
+        <v>43</v>
+      </c>
+      <c r="G8" t="s" s="0">
+        <v>52</v>
+      </c>
       <c r="H8" t="s" s="0">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I8" t="s" s="0">
         <v>19</v>
@@ -548,26 +599,26 @@
     </row>
     <row r="9">
       <c r="A9" t="s" s="0">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B9" t="s" s="0">
         <v>34</v>
       </c>
       <c r="C9" t="s" s="0">
-        <v>23</v>
+        <v>55</v>
       </c>
       <c r="D9" t="s" s="0">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="E9" t="s" s="0">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="F9" t="s" s="0">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="G9" s="0"/>
       <c r="H9" t="s" s="0">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="I9" t="s" s="0">
         <v>19</v>
@@ -584,26 +635,26 @@
     </row>
     <row r="10">
       <c r="A10" t="s" s="0">
+        <v>59</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s" s="0">
         <v>55</v>
       </c>
-      <c r="B10" t="s" s="0">
-        <v>29</v>
-      </c>
-      <c r="C10" t="s" s="0">
+      <c r="D10" t="s" s="0">
         <v>56</v>
-      </c>
-      <c r="D10" t="s" s="0">
-        <v>57</v>
       </c>
       <c r="E10" t="s" s="0">
         <v>16</v>
       </c>
       <c r="F10" t="s" s="0">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G10" s="0"/>
       <c r="H10" t="s" s="0">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="I10" t="s" s="0">
         <v>19</v>
@@ -615,6 +666,152 @@
         <v>19</v>
       </c>
       <c r="L10" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>62</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="D11" t="s" s="0">
+        <v>64</v>
+      </c>
+      <c r="E11" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="F11" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="G11" s="0"/>
+      <c r="H11" t="s" s="0">
+        <v>66</v>
+      </c>
+      <c r="I11" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="J11" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="K11" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="L11" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>48</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>67</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="D12" t="s" s="0">
+        <v>68</v>
+      </c>
+      <c r="E12" t="s" s="0">
+        <v>30</v>
+      </c>
+      <c r="F12" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="G12" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="H12" t="s" s="0">
+        <v>70</v>
+      </c>
+      <c r="I12" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="J12" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="K12" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="L12" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>13</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="D13" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="E13" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="F13" t="s" s="0">
+        <v>73</v>
+      </c>
+      <c r="G13" s="0"/>
+      <c r="H13" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="I13" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="J13" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="K13" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="L13" t="s" s="0">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="D14" t="s" s="0">
+        <v>72</v>
+      </c>
+      <c r="E14" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="F14" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="G14" s="0"/>
+      <c r="H14" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="I14" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="J14" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="K14" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="L14" t="s" s="0">
         <v>20</v>
       </c>
     </row>

</xml_diff>